<commit_message>
commit d'Aloïs le main fonctionne !!! 15h42 19/06
</commit_message>
<xml_diff>
--- a/data/output/Garches_Equipe_3_feuille.xlsx
+++ b/data/output/Garches_Equipe_3_feuille.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,209 +425,120 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>type</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>geometry/type</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>longitude</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>latitude</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>intersection</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Ville/Commune</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Code Postale</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Code Département</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>Ville</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>Département</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ordre</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>nb_traversees</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>bande_de_guidage</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>bande_eveil</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>feu_parlant</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>commentaire</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>coordonnees</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Avenue  des  Jockeys  /  Allée  des  Jockeys</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Point</t>
+          <t>Garches, Hauts-de-Seine</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.202805027</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>48.851007576</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Avenue  des  Jockeys  /  Allée  des  Jockeys</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Garches, Hauts-de-Seine</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>92033</v>
-      </c>
-      <c r="H2" t="n">
-        <v>92</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Garches</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Hauts-de-Seine</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>3</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1</v>
-      </c>
-      <c r="M2" t="n">
-        <v>3</v>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
+          <t>48.851007576,2.202805027</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Feature</t>
+          <t>Avenue  des  Jockeys  /  Rue  de  Buzenval  D180</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Point</t>
+          <t>Garches, Hauts-de-Seine</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.203707677</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>48.852276402</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Avenue  des  Jockeys  /  Rue  de  Buzenval  D180</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Garches, Hauts-de-Seine</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>92033</v>
-      </c>
-      <c r="H3" t="n">
-        <v>92</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Garches</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Hauts-de-Seine</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
-        <v>3</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2</v>
-      </c>
-      <c r="M3" t="n">
-        <v>4</v>
-      </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+          <t>48.852276402,2.203707677</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Export.py changement et suppressions
</commit_message>
<xml_diff>
--- a/data/output/Garches_Equipe_3_feuille.xlsx
+++ b/data/output/Garches_Equipe_3_feuille.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I34"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,12 +469,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.841979871,2.196303482</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue  Jean  Mermoz  /  Avenue  Lyautey</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -494,12 +494,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.841979871,2.196303482</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue  Jean  Mermoz  /  Avenue  Lyautey</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -519,12 +519,12 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.841979871,2.196303482</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue  Jean  Mermoz  /  Avenue  Lyautey</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -544,19 +544,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.842952116,2.195521507</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Grande  Rue   /  Avenue  Lyautey</t>
         </is>
       </c>
       <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="n">
         <v>1</v>
-      </c>
-      <c r="E5" t="n">
-        <v>4</v>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
@@ -569,19 +569,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.842952116,2.195521507</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Grande  Rue   /  Avenue  Lyautey</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
@@ -594,19 +594,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.849009323,2.201078516</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue   du  19 Janvier  /  Avenue   du  Maréchal  Foch</t>
         </is>
       </c>
       <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
         <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>6</v>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
@@ -619,19 +619,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.849009323,2.201078516</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue   du  19 Janvier  /  Avenue   du  Maréchal  Foch</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
@@ -644,19 +644,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>48.82766635,2.275598465</t>
+          <t>48.849009323,2.201078516</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Boulevard  Gambetta  D50  /  Rue  Henri  Mayer</t>
+          <t>Rue   du  19 Janvier  /  Avenue   du  Maréchal  Foch</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
@@ -669,19 +669,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>48.827551946,2.276195745</t>
+          <t>48.849009323,2.201078516</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Rue  Vaudétard  Déviation D50  /  Boulevard  Gambetta  D50</t>
+          <t>Rue   du  19 Janvier  /  Avenue   du  Maréchal  Foch</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
@@ -694,19 +694,19 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>48.827551946,2.276195745</t>
+          <t>48.849009323,2.201078516</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rue  Vaudétard  Déviation D50  /  Boulevard  Gambetta  D50</t>
+          <t>Rue   du  19 Janvier  /  Avenue   du  Maréchal  Foch</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
@@ -719,19 +719,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>48.827551946,2.276195745</t>
+          <t>48.850268929,2.202306711</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Rue  Vaudétard  Déviation D50  /  Boulevard  Gambetta  D50</t>
+          <t>Avenue  des  Jockeys  /  Rue   du   Docteur   Debat</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E12" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
@@ -744,19 +744,19 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>48.827377989,2.277736531</t>
+          <t>48.850268929,2.202306711</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rue  Michel de  l'Hospital  /  Boulevard  Gambetta  D50</t>
+          <t>Avenue  des  Jockeys  /  Rue   du   Docteur   Debat</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
@@ -769,19 +769,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>48.827377989,2.277736531</t>
+          <t>48.850268929,2.202306711</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rue  Michel de  l'Hospital  /  Boulevard  Gambetta  D50</t>
+          <t>Avenue  des  Jockeys  /  Rue   du   Docteur   Debat</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
@@ -794,500 +794,25 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>48.827377989,2.277736531</t>
+          <t>48.850268929,2.202306711</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rue  Michel de  l'Hospital  /  Boulevard  Gambetta  D50</t>
+          <t>Avenue  des  Jockeys  /  Rue   du   Docteur   Debat</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
     </row>
-    <row r="16">
-      <c r="A16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>48.827241978,2.27850549</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Place  Paul  Vaillant-Couturier  D50  /  Boulevard  Gambetta  D50 / Rue  Ernest Renan  /  Boulevard  Gambetta  D50</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>4</v>
-      </c>
-      <c r="E16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>48.827241978,2.27850549</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Place  Paul  Vaillant-Couturier  D50  /  Boulevard  Gambetta  D50 / Rue  Ernest Renan  /  Boulevard  Gambetta  D50</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>4</v>
-      </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>48.827241978,2.27850549</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Place  Paul  Vaillant-Couturier  D50  /  Boulevard  Gambetta  D50 / Rue  Ernest Renan  /  Boulevard  Gambetta  D50</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" t="n">
-        <v>3</v>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>5</v>
-      </c>
-      <c r="E19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="n">
-        <v>3</v>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>5</v>
-      </c>
-      <c r="E20" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="n">
-        <v>3</v>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>5</v>
-      </c>
-      <c r="E21" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>3</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>5</v>
-      </c>
-      <c r="E22" t="n">
-        <v>4</v>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>3</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>5</v>
-      </c>
-      <c r="E23" t="n">
-        <v>5</v>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>3</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>48.826945349,2.279229322</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Place  Paul  Vaillant-Couturier  D50 / Boulevard  Voltaire  D50  /  Rue  Ernest Renan  D989 / Rue   du  Général  Leclerc  D989  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>5</v>
-      </c>
-      <c r="E24" t="n">
-        <v>6</v>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>3</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>48.825904897,2.280482734</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Rue  Voltaire  Déviation D50 / Rue  Voltaire  Déviation D50  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>6</v>
-      </c>
-      <c r="E25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>3</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>48.825904897,2.280482734</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Boulevard  Voltaire  D50  /  Rue  Voltaire  Déviation D50 / Rue  Voltaire  Déviation D50  /  Boulevard  Voltaire  D50</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>6</v>
-      </c>
-      <c r="E26" t="n">
-        <v>2</v>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>48.823000322,2.276203658</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Place  de  l'Église  /  Avenue  Jean  Jaurès / Rue  Minard  /  Avenue  Jean  Jaurès</t>
-        </is>
-      </c>
-      <c r="D27" t="n">
-        <v>8</v>
-      </c>
-      <c r="E27" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr"/>
-      <c r="I27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>3</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>48.823000322,2.276203658</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Place  de  l'Église  /  Avenue  Jean  Jaurès / Rue  Minard  /  Avenue  Jean  Jaurès</t>
-        </is>
-      </c>
-      <c r="D28" t="n">
-        <v>8</v>
-      </c>
-      <c r="E28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>3</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>48.823000322,2.276203658</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Place  de  l'Église  /  Avenue  Jean  Jaurès / Rue  Minard  /  Avenue  Jean  Jaurès</t>
-        </is>
-      </c>
-      <c r="D29" t="n">
-        <v>8</v>
-      </c>
-      <c r="E29" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>3</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>48.823000322,2.276203658</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Place  de  l'Église  /  Avenue  Jean  Jaurès / Rue  Minard  /  Avenue  Jean  Jaurès</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>8</v>
-      </c>
-      <c r="E30" t="n">
-        <v>4</v>
-      </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
-      <c r="H30" t="inlineStr"/>
-      <c r="I30" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>3</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>48.823000322,2.276203658</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Place  de  l'Église  /  Avenue  Jean  Jaurès / Rue  Minard  /  Avenue  Jean  Jaurès</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>8</v>
-      </c>
-      <c r="E31" t="n">
-        <v>5</v>
-      </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>3</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>48.830454422,2.284874085</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Rue   du  Quatre Septembre  /  Avenue  Ernest Renan / Rue   du  Quatre Septembre  /  Boulevard  Périphérique Extérieur / Rue  Ernest Renan  D989  /  Avenue  Ernest Renan</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>9</v>
-      </c>
-      <c r="E32" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>3</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>48.830454422,2.284874085</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Rue   du  Quatre Septembre  /  Avenue  Ernest Renan / Rue   du  Quatre Septembre  /  Boulevard  Périphérique Extérieur / Rue  Ernest Renan  D989  /  Avenue  Ernest Renan</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>9</v>
-      </c>
-      <c r="E33" t="n">
-        <v>2</v>
-      </c>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>3</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>48.830454422,2.284874085</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Rue   du  Quatre Septembre  /  Avenue  Ernest Renan / Rue   du  Quatre Septembre  /  Boulevard  Périphérique Extérieur / Rue  Ernest Renan  D989  /  Avenue  Ernest Renan</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>9</v>
-      </c>
-      <c r="E34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>